<commit_message>
Admin update: Configurator Data (Parts and Presets updated)
</commit_message>
<xml_diff>
--- a/Configurator_Data.xlsx
+++ b/Configurator_Data.xlsx
@@ -598,7 +598,7 @@
         <v>BLK-SG</v>
       </c>
       <c r="G3" t="str">
-        <v>XXXX</v>
+        <v>1999</v>
       </c>
       <c r="H3" t="str">
         <v>available</v>
@@ -627,7 +627,7 @@
         <v>WB-1330</v>
       </c>
       <c r="G4" t="str">
-        <v>XXXX</v>
+        <v>999</v>
       </c>
       <c r="H4" t="str">
         <v>available</v>
@@ -656,7 +656,7 @@
         <v>MOT-A-1330</v>
       </c>
       <c r="G5" t="str">
-        <v>XXXX</v>
+        <v>999</v>
       </c>
       <c r="H5" t="str">
         <v>available</v>
@@ -714,7 +714,7 @@
         <v>CTL-COL</v>
       </c>
       <c r="G7" t="str">
-        <v>XXX</v>
+        <v>500</v>
       </c>
       <c r="H7" t="str">
         <v>available</v>
@@ -743,7 +743,7 @@
         <v>CTL-HBAR</v>
       </c>
       <c r="G8" t="str">
-        <v>XXX</v>
+        <v>500</v>
       </c>
       <c r="H8" t="str">
         <v>available</v>
@@ -898,7 +898,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:I13"/>
   </ignoredErrors>
@@ -1166,13 +1165,19 @@
       <c r="J3" t="str">
         <v>body-sidesteplg, body-fenders, body-frontbumper, body-rearbumper</v>
       </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
         <v>Essential</v>
       </c>
       <c r="B4" t="str">
-        <v>Basic configuration</v>
+        <v>Basic Urban Mobility</v>
       </c>
       <c r="C4" t="str">
         <v>block-single</v>

</xml_diff>

<commit_message>
Admin update: Configurator Data (Parts, Presets, Categories updated)
</commit_message>
<xml_diff>
--- a/Configurator_Data.xlsx
+++ b/Configurator_Data.xlsx
@@ -551,80 +551,80 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Category name (must match Categories sheet)</v>
+        <v>Block</v>
       </c>
       <c r="B2" t="str">
-        <v>Display name shown to users</v>
+        <v>Single Block</v>
       </c>
       <c r="C2" t="str">
-        <v>Unique ID (auto-generated if blank)</v>
+        <v>block-single</v>
       </c>
       <c r="D2" t="str">
-        <v>GLB filename containing this part</v>
+        <v>block.glb</v>
       </c>
       <c r="E2" t="str">
-        <v>Exact node name inside the GLB file</v>
+        <v>Block_Single</v>
       </c>
       <c r="F2" t="str">
-        <v>Shopify/Inventory SKU code</v>
+        <v>BLK-SG</v>
       </c>
       <c r="G2" t="str">
-        <v>Price in default currency</v>
+        <v>1999</v>
       </c>
       <c r="H2" t="str">
-        <v>available / coming_soon / discontinued</v>
+        <v>available</v>
       </c>
       <c r="I2" t="str">
-        <v>Optional description for tooltips</v>
+        <v>Single width chassis block</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Block</v>
+        <v>Wheelbase</v>
       </c>
       <c r="B3" t="str">
-        <v>Single Block</v>
+        <v>Long Wheelbase 1330</v>
       </c>
       <c r="C3" t="str">
-        <v>block-single</v>
+        <v>wb-1330</v>
       </c>
       <c r="D3" t="str">
-        <v>block.glb</v>
+        <v>wb.glb</v>
       </c>
       <c r="E3" t="str">
-        <v>Block_Single</v>
+        <v>WB_1330</v>
       </c>
       <c r="F3" t="str">
-        <v>BLK-SG</v>
+        <v>WB-1330</v>
       </c>
       <c r="G3" t="str">
-        <v>1999</v>
+        <v>999</v>
       </c>
       <c r="H3" t="str">
         <v>available</v>
       </c>
       <c r="I3" t="str">
-        <v>Single width chassis block</v>
+        <v xml:space="preserve">long wheelbase </v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Wheelbase</v>
+        <v>Motor</v>
       </c>
       <c r="B4" t="str">
-        <v>Long Wheelbase 1330</v>
+        <v>Motor A 1330</v>
       </c>
       <c r="C4" t="str">
-        <v>wb-1330</v>
+        <v>motor-a-1330</v>
       </c>
       <c r="D4" t="str">
-        <v>wb.glb</v>
+        <v>motor.glb</v>
       </c>
       <c r="E4" t="str">
-        <v>WB_1330</v>
+        <v>Motor_A_1330</v>
       </c>
       <c r="F4" t="str">
-        <v>WB-1330</v>
+        <v>MOT-A-1330</v>
       </c>
       <c r="G4" t="str">
         <v>999</v>
@@ -633,65 +633,65 @@
         <v>available</v>
       </c>
       <c r="I4" t="str">
-        <v xml:space="preserve">long wheelbase </v>
+        <v>Motor Type A For short wheelbase</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Motor</v>
+        <v>Tire</v>
       </c>
       <c r="B5" t="str">
-        <v>Motor A 1330</v>
+        <v>Offroad Tires 1330</v>
       </c>
       <c r="C5" t="str">
-        <v>motor-a-1330</v>
+        <v>tire-offroad-1330</v>
       </c>
       <c r="D5" t="str">
-        <v>motor.glb</v>
+        <v>tire.glb</v>
       </c>
       <c r="E5" t="str">
-        <v>Motor_A_1330</v>
+        <v>Tire_Offroad_1330</v>
       </c>
       <c r="F5" t="str">
-        <v>MOT-A-1330</v>
-      </c>
-      <c r="G5" t="str">
-        <v>999</v>
+        <v>TIRE-OFF-1330</v>
+      </c>
+      <c r="G5">
+        <v>549</v>
       </c>
       <c r="H5" t="str">
         <v>available</v>
       </c>
       <c r="I5" t="str">
-        <v>Motor Type A For short wheelbase</v>
+        <v xml:space="preserve">All-terrain tires for Long wheelbase </v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Tire</v>
+        <v>Control</v>
       </c>
       <c r="B6" t="str">
-        <v>Offroad Tires 1330</v>
+        <v>Column Standard Position</v>
       </c>
       <c r="C6" t="str">
-        <v>tire-offroad-1330</v>
+        <v>control-column</v>
       </c>
       <c r="D6" t="str">
-        <v>tire.glb</v>
+        <v>control.glb</v>
       </c>
       <c r="E6" t="str">
-        <v>Tire_Offroad_1330</v>
+        <v>Control_Column</v>
       </c>
       <c r="F6" t="str">
-        <v>TIRE-OFF-1330</v>
-      </c>
-      <c r="G6">
-        <v>549</v>
+        <v>CTL-COL</v>
+      </c>
+      <c r="G6" t="str">
+        <v>500</v>
       </c>
       <c r="H6" t="str">
         <v>available</v>
       </c>
       <c r="I6" t="str">
-        <v xml:space="preserve">All-terrain tires for Long wheelbase </v>
+        <v>Standard Column</v>
       </c>
     </row>
     <row r="7">
@@ -699,19 +699,19 @@
         <v>Control</v>
       </c>
       <c r="B7" t="str">
-        <v>Column Standard Position</v>
+        <v>Handle Bar</v>
       </c>
       <c r="C7" t="str">
-        <v>control-column</v>
+        <v>control-handlebar</v>
       </c>
       <c r="D7" t="str">
         <v>control.glb</v>
       </c>
       <c r="E7" t="str">
-        <v>Control_Column</v>
+        <v>Control_Handlebar</v>
       </c>
       <c r="F7" t="str">
-        <v>CTL-COL</v>
+        <v>CTL-HBAR</v>
       </c>
       <c r="G7" t="str">
         <v>500</v>
@@ -720,65 +720,65 @@
         <v>available</v>
       </c>
       <c r="I7" t="str">
-        <v>Standard Column</v>
+        <v>Standard Handle Bar</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Control</v>
+        <v>Seat</v>
       </c>
       <c r="B8" t="str">
-        <v>Handle Bar</v>
+        <v>Leaning Seat</v>
       </c>
       <c r="C8" t="str">
-        <v>control-handlebar</v>
+        <v>seat-leaning</v>
       </c>
       <c r="D8" t="str">
-        <v>control.glb</v>
+        <v>seat.glb</v>
       </c>
       <c r="E8" t="str">
-        <v>Control_Handlebar</v>
+        <v>Seat_Leaning</v>
       </c>
       <c r="F8" t="str">
-        <v>CTL-HBAR</v>
-      </c>
-      <c r="G8" t="str">
-        <v>500</v>
+        <v>SEAT-LEAN</v>
+      </c>
+      <c r="G8">
+        <v>299</v>
       </c>
       <c r="H8" t="str">
         <v>available</v>
       </c>
       <c r="I8" t="str">
-        <v>Standard Handle Bar</v>
+        <v>Compact standing/leaning seat</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Seat</v>
+        <v>Body</v>
       </c>
       <c r="B9" t="str">
-        <v>Leaning Seat</v>
+        <v>Side Steps Large</v>
       </c>
       <c r="C9" t="str">
-        <v>seat-leaning</v>
+        <v>body-sidesteplg</v>
       </c>
       <c r="D9" t="str">
-        <v>seat.glb</v>
+        <v>body.glb</v>
       </c>
       <c r="E9" t="str">
-        <v>Seat_Leaning</v>
+        <v>Body_SideStepLg</v>
       </c>
       <c r="F9" t="str">
-        <v>SEAT-LEAN</v>
+        <v>BODY-STEPL</v>
       </c>
       <c r="G9">
-        <v>299</v>
+        <v>249</v>
       </c>
       <c r="H9" t="str">
         <v>available</v>
       </c>
       <c r="I9" t="str">
-        <v>Compact standing/leaning seat</v>
+        <v>Foot side steps Large</v>
       </c>
     </row>
     <row r="10">
@@ -786,28 +786,28 @@
         <v>Body</v>
       </c>
       <c r="B10" t="str">
-        <v>Side Steps Large</v>
+        <v>Fenders</v>
       </c>
       <c r="C10" t="str">
-        <v>body-sidesteplg</v>
+        <v>body-fenders</v>
       </c>
       <c r="D10" t="str">
         <v>body.glb</v>
       </c>
       <c r="E10" t="str">
-        <v>Body_SideStepLg</v>
+        <v>Body_Fenders</v>
       </c>
       <c r="F10" t="str">
-        <v>BODY-STEPL</v>
+        <v>BODY-FEND</v>
       </c>
       <c r="G10">
-        <v>249</v>
+        <v>179</v>
       </c>
       <c r="H10" t="str">
         <v>available</v>
       </c>
       <c r="I10" t="str">
-        <v>Foot side steps Large</v>
+        <v>Wheel fenders</v>
       </c>
     </row>
     <row r="11">
@@ -815,28 +815,28 @@
         <v>Body</v>
       </c>
       <c r="B11" t="str">
-        <v>Fenders</v>
+        <v>Front Bumper</v>
       </c>
       <c r="C11" t="str">
-        <v>body-fenders</v>
+        <v>body-frontbumper</v>
       </c>
       <c r="D11" t="str">
         <v>body.glb</v>
       </c>
       <c r="E11" t="str">
-        <v>Body_Fenders</v>
+        <v>Body_FrontBumper</v>
       </c>
       <c r="F11" t="str">
-        <v>BODY-FEND</v>
+        <v>BODY-FBUMP</v>
       </c>
       <c r="G11">
-        <v>179</v>
+        <v>299</v>
       </c>
       <c r="H11" t="str">
         <v>available</v>
       </c>
       <c r="I11" t="str">
-        <v>Wheel fenders</v>
+        <v>Multifunctional front bumper</v>
       </c>
     </row>
     <row r="12">
@@ -844,19 +844,19 @@
         <v>Body</v>
       </c>
       <c r="B12" t="str">
-        <v>Front Bumper</v>
+        <v>Rear Bumper</v>
       </c>
       <c r="C12" t="str">
-        <v>body-frontbumper</v>
+        <v>body-rearbumper</v>
       </c>
       <c r="D12" t="str">
         <v>body.glb</v>
       </c>
       <c r="E12" t="str">
-        <v>Body_FrontBumper</v>
+        <v>Body_RearBumper</v>
       </c>
       <c r="F12" t="str">
-        <v>BODY-FBUMP</v>
+        <v>BODY-RBUMP</v>
       </c>
       <c r="G12">
         <v>299</v>
@@ -865,36 +865,30 @@
         <v>available</v>
       </c>
       <c r="I12" t="str">
-        <v>Multifunctional front bumper</v>
+        <v>Multifunctional rear bumper</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Body</v>
+        <v>Wheelbase</v>
       </c>
       <c r="B13" t="str">
-        <v>Rear Bumper</v>
+        <v>Short Wheelbase 1130</v>
       </c>
       <c r="C13" t="str">
-        <v>body-rearbumper</v>
+        <v>wb-1130</v>
       </c>
       <c r="D13" t="str">
-        <v>body.glb</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Body_RearBumper</v>
+        <v>models/parts/placeholder.glb</v>
       </c>
       <c r="F13" t="str">
-        <v>BODY-RBUMP</v>
-      </c>
-      <c r="G13">
-        <v>299</v>
+        <v>SKU-000</v>
+      </c>
+      <c r="G13" t="str">
+        <v>999</v>
       </c>
       <c r="H13" t="str">
-        <v>available</v>
-      </c>
-      <c r="I13" t="str">
-        <v>Multifunctional rear bumper</v>
+        <v>active</v>
       </c>
     </row>
   </sheetData>
@@ -1181,7 +1175,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1205,30 +1199,30 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Category name (must match Parts sheet)</v>
+        <v>Block</v>
       </c>
       <c r="B2" t="str">
-        <v>Name shown in UI</v>
+        <v>Chassis</v>
       </c>
       <c r="C2" t="str">
-        <v>single (pick one) or multi (pick many)</v>
-      </c>
-      <c r="D2" t="str">
-        <v>1=load first (base), 2+=lazy load</v>
+        <v>single</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
       </c>
       <c r="E2" t="str">
-        <v>yes/no - must user select?</v>
+        <v>yes</v>
       </c>
       <c r="F2" t="str">
-        <v>Optional icon name</v>
+        <v>chassis</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Block</v>
+        <v>Wheelbase</v>
       </c>
       <c r="B3" t="str">
-        <v>Chassis</v>
+        <v>Wheelbase</v>
       </c>
       <c r="C3" t="str">
         <v>single</v>
@@ -1240,15 +1234,15 @@
         <v>yes</v>
       </c>
       <c r="F3" t="str">
-        <v>chassis</v>
+        <v>wheelbase</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Wheelbase</v>
+        <v>Motor</v>
       </c>
       <c r="B4" t="str">
-        <v>Wheelbase</v>
+        <v>Electric Motor</v>
       </c>
       <c r="C4" t="str">
         <v>single</v>
@@ -1260,15 +1254,15 @@
         <v>yes</v>
       </c>
       <c r="F4" t="str">
-        <v>wheelbase</v>
+        <v>motor</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Motor</v>
+        <v>Tire</v>
       </c>
       <c r="B5" t="str">
-        <v>Electric Motor</v>
+        <v>Wheels &amp; Tires</v>
       </c>
       <c r="C5" t="str">
         <v>single</v>
@@ -1280,35 +1274,35 @@
         <v>yes</v>
       </c>
       <c r="F5" t="str">
-        <v>motor</v>
+        <v>tire</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Tire</v>
+        <v>Control</v>
       </c>
       <c r="B6" t="str">
-        <v>Wheels &amp; Tires</v>
+        <v>Steering Control</v>
       </c>
       <c r="C6" t="str">
         <v>single</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" t="str">
         <v>yes</v>
       </c>
       <c r="F6" t="str">
-        <v>tire</v>
+        <v>control</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Control</v>
+        <v>Seat</v>
       </c>
       <c r="B7" t="str">
-        <v>Steering Control</v>
+        <v>Seating</v>
       </c>
       <c r="C7" t="str">
         <v>single</v>
@@ -1320,93 +1314,72 @@
         <v>yes</v>
       </c>
       <c r="F7" t="str">
-        <v>control</v>
+        <v>seat</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Seat</v>
+        <v>Body</v>
       </c>
       <c r="B8" t="str">
-        <v>Seating</v>
+        <v>Body Parts</v>
       </c>
       <c r="C8" t="str">
-        <v>single</v>
+        <v>multi</v>
       </c>
       <c r="D8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E8" t="str">
-        <v>yes</v>
+        <v>no</v>
       </c>
       <c r="F8" t="str">
-        <v>seat</v>
+        <v>body</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Body</v>
+        <v>Accessories</v>
       </c>
       <c r="B9" t="str">
-        <v>Body Parts</v>
+        <v>Accessories</v>
       </c>
       <c r="C9" t="str">
         <v>multi</v>
       </c>
       <c r="D9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E9" t="str">
         <v>no</v>
       </c>
       <c r="F9" t="str">
-        <v>body</v>
+        <v>accessories</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Accessories</v>
+        <v>Color</v>
       </c>
       <c r="B10" t="str">
-        <v>Accessories</v>
+        <v>Color &amp; Finish</v>
       </c>
       <c r="C10" t="str">
-        <v>multi</v>
+        <v>single</v>
       </c>
       <c r="D10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E10" t="str">
         <v>no</v>
       </c>
       <c r="F10" t="str">
-        <v>accessories</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Color</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Color &amp; Finish</v>
-      </c>
-      <c r="C11" t="str">
-        <v>single</v>
-      </c>
-      <c r="D11">
-        <v>5</v>
-      </c>
-      <c r="E11" t="str">
-        <v>no</v>
-      </c>
-      <c r="F11" t="str">
         <v>palette</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix: Sync 1130 wheelbase rendering and rules to source Excel and add placeholder GLB
</commit_message>
<xml_diff>
--- a/Configurator_Data.xlsx
+++ b/Configurator_Data.xlsx
@@ -518,7 +518,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -879,10 +879,10 @@
         <v>wb-1130</v>
       </c>
       <c r="D13" t="str">
-        <v>models/parts/placeholder.glb</v>
+        <v>wb.glb</v>
       </c>
       <c r="E13" t="str">
-        <v/>
+        <v>WB_1130</v>
       </c>
       <c r="F13" t="str">
         <v>SKU-000</v>
@@ -897,16 +897,74 @@
         <v/>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Motor</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Motor A 1130</v>
+      </c>
+      <c r="C14" t="str">
+        <v>motor-a-1130</v>
+      </c>
+      <c r="D14" t="str">
+        <v>motor.glb</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Motor_A_1130</v>
+      </c>
+      <c r="F14" t="str">
+        <v>MOT-A-1130</v>
+      </c>
+      <c r="G14">
+        <v>899</v>
+      </c>
+      <c r="H14" t="str">
+        <v>available</v>
+      </c>
+      <c r="I14" t="str">
+        <v>Motor Type A for Short wheelbase</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Tire</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Offroad Tires 1130</v>
+      </c>
+      <c r="C15" t="str">
+        <v>tire-offroad-1130</v>
+      </c>
+      <c r="D15" t="str">
+        <v>tire.glb</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Tire_Offroad_1130</v>
+      </c>
+      <c r="F15" t="str">
+        <v>TIRE-OFF-1130</v>
+      </c>
+      <c r="G15">
+        <v>499</v>
+      </c>
+      <c r="H15" t="str">
+        <v>available</v>
+      </c>
+      <c r="I15" t="str">
+        <v>All-terrain tires for Short wheelbase</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I15"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1046,10 +1104,51 @@
         <v>block-single</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>wb-1130</v>
+      </c>
+      <c r="B13" t="str">
+        <v>REQUIRES</v>
+      </c>
+      <c r="C13" t="str">
+        <v>block-single</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>motor-a-1130</v>
+      </c>
+      <c r="B14" t="str">
+        <v>REQUIRES</v>
+      </c>
+      <c r="C14" t="str">
+        <v>wb-1130</v>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>tire-offroad-1130</v>
+      </c>
+      <c r="B15" t="str">
+        <v>REQUIRES</v>
+      </c>
+      <c r="C15" t="str">
+        <v>motor-a-1130</v>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix: Re-add handlebar and remove conflicting REQUIRES rule to enable selection
</commit_message>
<xml_diff>
--- a/Configurator_Data.xlsx
+++ b/Configurator_Data.xlsx
@@ -713,7 +713,7 @@
       <c r="F7" t="str">
         <v>CTL-HBAR</v>
       </c>
-      <c r="G7" t="str">
+      <c r="G7">
         <v>500</v>
       </c>
       <c r="H7" t="str">
@@ -964,7 +964,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1040,18 +1040,18 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>control-handlebar</v>
+        <v>seat-leaning</v>
       </c>
       <c r="B7" t="str">
         <v>REQUIRES</v>
       </c>
       <c r="C7" t="str">
-        <v>control-column</v>
+        <v>block-single</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>seat-leaning</v>
+        <v>body-sidesteplg</v>
       </c>
       <c r="B8" t="str">
         <v>REQUIRES</v>
@@ -1062,7 +1062,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>body-sidesteplg</v>
+        <v>body-fenders</v>
       </c>
       <c r="B9" t="str">
         <v>REQUIRES</v>
@@ -1073,7 +1073,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>body-fenders</v>
+        <v>body-frontbumper</v>
       </c>
       <c r="B10" t="str">
         <v>REQUIRES</v>
@@ -1084,7 +1084,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>body-frontbumper</v>
+        <v>body-rearbumper</v>
       </c>
       <c r="B11" t="str">
         <v>REQUIRES</v>
@@ -1095,7 +1095,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>body-rearbumper</v>
+        <v>wb-1130</v>
       </c>
       <c r="B12" t="str">
         <v>REQUIRES</v>
@@ -1103,16 +1103,19 @@
       <c r="C12" t="str">
         <v>block-single</v>
       </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>wb-1130</v>
+        <v>motor-a-1130</v>
       </c>
       <c r="B13" t="str">
         <v>REQUIRES</v>
       </c>
       <c r="C13" t="str">
-        <v>block-single</v>
+        <v>wb-1130</v>
       </c>
       <c r="D13" t="str">
         <v/>
@@ -1120,35 +1123,21 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>motor-a-1130</v>
+        <v>tire-offroad-1130</v>
       </c>
       <c r="B14" t="str">
         <v>REQUIRES</v>
       </c>
       <c r="C14" t="str">
-        <v>wb-1130</v>
+        <v>motor-a-1130</v>
       </c>
       <c r="D14" t="str">
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>tire-offroad-1130</v>
-      </c>
-      <c r="B15" t="str">
-        <v>REQUIRES</v>
-      </c>
-      <c r="C15" t="str">
-        <v>motor-a-1130</v>
-      </c>
-      <c r="D15" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D14"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix leaning seat GLB node (Seat_Leaning), aliases, safer UPTModel visibility
- Map Leaning_Seat to Seat_Leaning via nodeNameAliases.json
- Apply aliases in processNewData; resolve at runtime in UPTModel
- Remove show-all-GLB fallback on unknown nodes (warn instead)
- Regenerate configMatrix from workbook

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Configurator_Data.xlsx
+++ b/Configurator_Data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samrosati/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samrosati/Documents/upt-configurator-test-repo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E3CFB0D4-772F-F544-B67D-85BF3099355A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{634E7B65-7A0D-C243-8B75-21442EBD5191}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="640" yWindow="760" windowWidth="29320" windowHeight="18880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -858,9 +858,6 @@
     <t>Standup riding lean pad</t>
   </si>
   <si>
-    <t>Leaning_Seat</t>
-  </si>
-  <si>
     <t>seat-lean</t>
   </si>
   <si>
@@ -1150,6 +1147,9 @@
   </si>
   <si>
     <t>Gas and Brake Pedal set for Steering Wheel driving</t>
+  </si>
+  <si>
+    <t>Seat_Leaning</t>
   </si>
 </sst>
 </file>
@@ -1831,7 +1831,7 @@
         <v>40</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
@@ -1851,7 +1851,7 @@
         <v>149</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="G4" s="5">
         <v>999</v>
@@ -1880,7 +1880,7 @@
         <v>122</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="G5" s="5">
         <v>999</v>
@@ -1909,7 +1909,7 @@
         <v>153</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="G6" s="5">
         <v>999</v>
@@ -1938,7 +1938,7 @@
         <v>115</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="G7" s="5">
         <v>999</v>
@@ -1967,7 +1967,7 @@
         <v>157</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="G8" s="5">
         <v>399</v>
@@ -1996,7 +1996,7 @@
         <v>161</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="G9" s="5">
         <v>399</v>
@@ -2025,7 +2025,7 @@
         <v>165</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="G10" s="5">
         <v>399</v>
@@ -2054,7 +2054,7 @@
         <v>131</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="G11" s="5">
         <v>399</v>
@@ -2071,19 +2071,19 @@
         <v>102</v>
       </c>
       <c r="B12" s="5" t="s">
+        <v>361</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>362</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>363</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>130</v>
       </c>
       <c r="E12" s="5" t="s">
+        <v>363</v>
+      </c>
+      <c r="F12" s="5" t="s">
         <v>364</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>365</v>
       </c>
       <c r="G12" s="5">
         <v>399</v>
@@ -2113,7 +2113,7 @@
         <v>226</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="G13" s="5">
         <v>699</v>
@@ -2142,7 +2142,7 @@
         <v>231</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="G14" s="5">
         <v>699</v>
@@ -2171,7 +2171,7 @@
         <v>234</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="G15" s="5">
         <v>699</v>
@@ -2200,7 +2200,7 @@
         <v>227</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="G16" s="5">
         <v>699</v>
@@ -2217,19 +2217,19 @@
         <v>219</v>
       </c>
       <c r="B17" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>330</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>331</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>225</v>
       </c>
       <c r="E17" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="F17" s="5" t="s">
         <v>332</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>333</v>
       </c>
       <c r="G17" s="5">
         <v>699</v>
@@ -2238,7 +2238,7 @@
         <v>40</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="J17" s="11"/>
     </row>
@@ -2247,26 +2247,26 @@
         <v>219</v>
       </c>
       <c r="B18" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>335</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>336</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>225</v>
       </c>
       <c r="E18" s="5" t="s">
+        <v>336</v>
+      </c>
+      <c r="F18" s="5" t="s">
         <v>337</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>338</v>
       </c>
       <c r="G18" s="5"/>
       <c r="H18" s="5" t="s">
         <v>40</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="J18" s="11"/>
     </row>
@@ -2287,7 +2287,7 @@
         <v>266</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="G19" s="10">
         <v>499</v>
@@ -2316,7 +2316,7 @@
         <v>240</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="G20" s="10">
         <v>499</v>
@@ -2345,7 +2345,7 @@
         <v>244</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="G21" s="10">
         <v>499</v>
@@ -2374,7 +2374,7 @@
         <v>248</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="G22" s="10">
         <v>499</v>
@@ -2403,7 +2403,7 @@
         <v>250</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="G23" s="10">
         <v>699</v>
@@ -2432,7 +2432,7 @@
         <v>254</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="G24" s="10">
         <v>699</v>
@@ -2461,7 +2461,7 @@
         <v>261</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="G25" s="10">
         <v>699</v>
@@ -2478,26 +2478,26 @@
         <v>236</v>
       </c>
       <c r="B26" s="5" t="s">
+        <v>365</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>366</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>367</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>239</v>
       </c>
       <c r="E26" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="F26" s="5" t="s">
         <v>368</v>
-      </c>
-      <c r="F26" s="5" t="s">
-        <v>369</v>
       </c>
       <c r="G26" s="10"/>
       <c r="H26" s="5" t="s">
         <v>40</v>
       </c>
       <c r="I26" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="J26" s="11"/>
     </row>
@@ -2506,19 +2506,19 @@
         <v>236</v>
       </c>
       <c r="B27" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="C27" s="5" t="s">
         <v>340</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>341</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>239</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="G27" s="5">
         <v>699</v>
@@ -2527,7 +2527,7 @@
         <v>40</v>
       </c>
       <c r="I27" s="5" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="J27" s="11"/>
     </row>
@@ -2536,26 +2536,26 @@
         <v>236</v>
       </c>
       <c r="B28" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>344</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>345</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>239</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="G28" s="5"/>
       <c r="H28" s="5" t="s">
         <v>40</v>
       </c>
       <c r="I28" s="5" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="J28" s="11"/>
     </row>
@@ -2567,13 +2567,13 @@
         <v>42</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>133</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>273</v>
+        <v>370</v>
       </c>
       <c r="F29" s="5" t="s">
         <v>44</v>
@@ -2643,7 +2643,7 @@
         <v>40</v>
       </c>
       <c r="I31" s="5" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
@@ -2651,19 +2651,19 @@
         <v>41</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>133</v>
       </c>
       <c r="E32" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="F32" s="5" t="s">
         <v>279</v>
-      </c>
-      <c r="F32" s="5" t="s">
-        <v>280</v>
       </c>
       <c r="G32" s="10">
         <v>599</v>
@@ -2672,7 +2672,7 @@
         <v>40</v>
       </c>
       <c r="I32" s="5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.2">
@@ -2680,19 +2680,19 @@
         <v>41</v>
       </c>
       <c r="B33" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="C33" s="5" t="s">
         <v>348</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>349</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>133</v>
       </c>
       <c r="E33" s="5" t="s">
+        <v>349</v>
+      </c>
+      <c r="F33" s="5" t="s">
         <v>350</v>
-      </c>
-      <c r="F33" s="5" t="s">
-        <v>351</v>
       </c>
       <c r="G33" s="5">
         <v>599</v>
@@ -2701,7 +2701,7 @@
         <v>40</v>
       </c>
       <c r="I33" s="5" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="J33" s="11"/>
     </row>
@@ -2710,26 +2710,26 @@
         <v>41</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>133</v>
       </c>
       <c r="E34" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="F34" s="5" t="s">
         <v>354</v>
-      </c>
-      <c r="F34" s="5" t="s">
-        <v>355</v>
       </c>
       <c r="G34" s="5"/>
       <c r="H34" s="5" t="s">
         <v>40</v>
       </c>
       <c r="I34" s="5" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="J34" s="11"/>
     </row>
@@ -2953,7 +2953,7 @@
         <v>54</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="G42" s="10">
         <v>299</v>
@@ -2982,7 +2982,7 @@
         <v>142</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="G43" s="10">
         <v>299</v>
@@ -3011,7 +3011,7 @@
         <v>202</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="G44" s="10">
         <v>299</v>
@@ -3040,7 +3040,7 @@
         <v>206</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="G45" s="10">
         <v>299</v>
@@ -3060,16 +3060,16 @@
         <v>269</v>
       </c>
       <c r="C46" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="D46" s="5" t="s">
         <v>283</v>
       </c>
-      <c r="D46" s="5" t="s">
+      <c r="E46" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="E46" s="5" t="s">
+      <c r="F46" s="5" t="s">
         <v>285</v>
-      </c>
-      <c r="F46" s="5" t="s">
-        <v>286</v>
       </c>
       <c r="G46" s="10">
         <v>2099</v>
@@ -3078,7 +3078,7 @@
         <v>40</v>
       </c>
       <c r="I46" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="J46" s="11"/>
     </row>
@@ -3090,16 +3090,16 @@
         <v>270</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="F47" s="5" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="G47" s="10">
         <v>3099</v>
@@ -3108,7 +3108,7 @@
         <v>40</v>
       </c>
       <c r="I47" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="J47" s="11"/>
     </row>
@@ -3120,16 +3120,16 @@
         <v>271</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="G48" s="5">
         <v>2399</v>
@@ -3138,7 +3138,7 @@
         <v>40</v>
       </c>
       <c r="I48" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J48" s="11"/>
     </row>
@@ -3147,19 +3147,19 @@
         <v>268</v>
       </c>
       <c r="B49" s="5" t="s">
+        <v>356</v>
+      </c>
+      <c r="C49" s="5" t="s">
         <v>357</v>
       </c>
-      <c r="C49" s="5" t="s">
+      <c r="D49" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="E49" s="5" t="s">
         <v>358</v>
       </c>
-      <c r="D49" s="5" t="s">
-        <v>284</v>
-      </c>
-      <c r="E49" s="5" t="s">
+      <c r="F49" s="5" t="s">
         <v>359</v>
-      </c>
-      <c r="F49" s="5" t="s">
-        <v>360</v>
       </c>
       <c r="G49" s="5">
         <v>2399</v>
@@ -3168,7 +3168,7 @@
         <v>40</v>
       </c>
       <c r="I49" s="5" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="J49" s="11"/>
     </row>
@@ -3235,19 +3235,19 @@
         <v>55</v>
       </c>
       <c r="B52" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="C52" s="5" t="s">
         <v>318</v>
       </c>
-      <c r="C52" s="5" t="s">
+      <c r="D52" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="E52" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="F52" s="5" t="s">
         <v>319</v>
-      </c>
-      <c r="D52" s="5" t="s">
-        <v>319</v>
-      </c>
-      <c r="E52" s="5" t="s">
-        <v>319</v>
-      </c>
-      <c r="F52" s="5" t="s">
-        <v>320</v>
       </c>
       <c r="G52" s="10">
         <v>1499</v>
@@ -3256,7 +3256,7 @@
         <v>40</v>
       </c>
       <c r="I52" s="5" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
   </sheetData>
@@ -3319,7 +3319,7 @@
         <v>148</v>
       </c>
       <c r="B4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C4" t="s">
         <v>112</v>
@@ -3341,7 +3341,7 @@
         <v>112</v>
       </c>
       <c r="B6" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C6" t="s">
         <v>148</v>
@@ -3363,7 +3363,7 @@
         <v>152</v>
       </c>
       <c r="B8" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C8" t="s">
         <v>125</v>
@@ -3385,7 +3385,7 @@
         <v>125</v>
       </c>
       <c r="B10" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C10" t="s">
         <v>152</v>
@@ -3407,7 +3407,7 @@
         <v>156</v>
       </c>
       <c r="B12" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C12" t="s">
         <v>160</v>
@@ -3418,7 +3418,7 @@
         <v>156</v>
       </c>
       <c r="B13" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C13" t="s">
         <v>164</v>
@@ -3429,7 +3429,7 @@
         <v>156</v>
       </c>
       <c r="B14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C14" t="s">
         <v>129</v>
@@ -3451,7 +3451,7 @@
         <v>160</v>
       </c>
       <c r="B16" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C16" t="s">
         <v>156</v>
@@ -3462,7 +3462,7 @@
         <v>160</v>
       </c>
       <c r="B17" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C17" t="s">
         <v>164</v>
@@ -3473,7 +3473,7 @@
         <v>160</v>
       </c>
       <c r="B18" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C18" t="s">
         <v>129</v>
@@ -3495,7 +3495,7 @@
         <v>164</v>
       </c>
       <c r="B20" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C20" t="s">
         <v>156</v>
@@ -3506,7 +3506,7 @@
         <v>164</v>
       </c>
       <c r="B21" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C21" t="s">
         <v>160</v>
@@ -3517,7 +3517,7 @@
         <v>164</v>
       </c>
       <c r="B22" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C22" t="s">
         <v>129</v>
@@ -3539,7 +3539,7 @@
         <v>129</v>
       </c>
       <c r="B24" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C24" t="s">
         <v>156</v>
@@ -3550,7 +3550,7 @@
         <v>129</v>
       </c>
       <c r="B25" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C25" t="s">
         <v>160</v>
@@ -3561,7 +3561,7 @@
         <v>129</v>
       </c>
       <c r="B26" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C26" t="s">
         <v>164</v>
@@ -3583,7 +3583,7 @@
         <v>222</v>
       </c>
       <c r="B28" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C28" t="s">
         <v>230</v>
@@ -3594,7 +3594,7 @@
         <v>222</v>
       </c>
       <c r="B29" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C29" t="s">
         <v>233</v>
@@ -3605,7 +3605,7 @@
         <v>222</v>
       </c>
       <c r="B30" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C30" t="s">
         <v>223</v>
@@ -3616,7 +3616,7 @@
         <v>222</v>
       </c>
       <c r="B31" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C31" t="s">
         <v>224</v>
@@ -3638,7 +3638,7 @@
         <v>230</v>
       </c>
       <c r="B33" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C33" t="s">
         <v>222</v>
@@ -3649,7 +3649,7 @@
         <v>230</v>
       </c>
       <c r="B34" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C34" t="s">
         <v>233</v>
@@ -3660,7 +3660,7 @@
         <v>230</v>
       </c>
       <c r="B35" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C35" t="s">
         <v>223</v>
@@ -3671,7 +3671,7 @@
         <v>230</v>
       </c>
       <c r="B36" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C36" t="s">
         <v>224</v>
@@ -3693,7 +3693,7 @@
         <v>233</v>
       </c>
       <c r="B38" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C38" t="s">
         <v>222</v>
@@ -3704,7 +3704,7 @@
         <v>233</v>
       </c>
       <c r="B39" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C39" t="s">
         <v>230</v>
@@ -3715,7 +3715,7 @@
         <v>233</v>
       </c>
       <c r="B40" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C40" t="s">
         <v>223</v>
@@ -3726,7 +3726,7 @@
         <v>233</v>
       </c>
       <c r="B41" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C41" t="s">
         <v>224</v>
@@ -3748,7 +3748,7 @@
         <v>223</v>
       </c>
       <c r="B43" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C43" t="s">
         <v>222</v>
@@ -3759,7 +3759,7 @@
         <v>223</v>
       </c>
       <c r="B44" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C44" t="s">
         <v>230</v>
@@ -3770,7 +3770,7 @@
         <v>223</v>
       </c>
       <c r="B45" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C45" t="s">
         <v>233</v>
@@ -3781,7 +3781,7 @@
         <v>223</v>
       </c>
       <c r="B46" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C46" t="s">
         <v>224</v>
@@ -3803,7 +3803,7 @@
         <v>224</v>
       </c>
       <c r="B48" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C48" t="s">
         <v>222</v>
@@ -3814,7 +3814,7 @@
         <v>224</v>
       </c>
       <c r="B49" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C49" t="s">
         <v>230</v>
@@ -3825,7 +3825,7 @@
         <v>224</v>
       </c>
       <c r="B50" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C50" t="s">
         <v>233</v>
@@ -3836,7 +3836,7 @@
         <v>224</v>
       </c>
       <c r="B51" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C51" t="s">
         <v>223</v>
@@ -3858,7 +3858,7 @@
         <v>264</v>
       </c>
       <c r="B53" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C53" t="s">
         <v>238</v>
@@ -3869,7 +3869,7 @@
         <v>264</v>
       </c>
       <c r="B54" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C54" t="s">
         <v>243</v>
@@ -3880,7 +3880,7 @@
         <v>264</v>
       </c>
       <c r="B55" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C55" t="s">
         <v>247</v>
@@ -3891,7 +3891,7 @@
         <v>264</v>
       </c>
       <c r="B56" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C56" t="s">
         <v>252</v>
@@ -3902,7 +3902,7 @@
         <v>264</v>
       </c>
       <c r="B57" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C57" t="s">
         <v>253</v>
@@ -3913,7 +3913,7 @@
         <v>264</v>
       </c>
       <c r="B58" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C58" t="s">
         <v>260</v>
@@ -3935,7 +3935,7 @@
         <v>238</v>
       </c>
       <c r="B60" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C60" t="s">
         <v>264</v>
@@ -3946,7 +3946,7 @@
         <v>238</v>
       </c>
       <c r="B61" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C61" t="s">
         <v>243</v>
@@ -3957,7 +3957,7 @@
         <v>238</v>
       </c>
       <c r="B62" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C62" t="s">
         <v>247</v>
@@ -3968,7 +3968,7 @@
         <v>238</v>
       </c>
       <c r="B63" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C63" t="s">
         <v>252</v>
@@ -3979,7 +3979,7 @@
         <v>238</v>
       </c>
       <c r="B64" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C64" t="s">
         <v>253</v>
@@ -3990,7 +3990,7 @@
         <v>238</v>
       </c>
       <c r="B65" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C65" t="s">
         <v>260</v>
@@ -4012,7 +4012,7 @@
         <v>243</v>
       </c>
       <c r="B67" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C67" t="s">
         <v>264</v>
@@ -4023,7 +4023,7 @@
         <v>243</v>
       </c>
       <c r="B68" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C68" t="s">
         <v>238</v>
@@ -4034,7 +4034,7 @@
         <v>243</v>
       </c>
       <c r="B69" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C69" t="s">
         <v>247</v>
@@ -4045,7 +4045,7 @@
         <v>243</v>
       </c>
       <c r="B70" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C70" t="s">
         <v>252</v>
@@ -4056,7 +4056,7 @@
         <v>243</v>
       </c>
       <c r="B71" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C71" t="s">
         <v>253</v>
@@ -4067,7 +4067,7 @@
         <v>243</v>
       </c>
       <c r="B72" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C72" t="s">
         <v>260</v>
@@ -4089,7 +4089,7 @@
         <v>247</v>
       </c>
       <c r="B74" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C74" t="s">
         <v>264</v>
@@ -4100,7 +4100,7 @@
         <v>247</v>
       </c>
       <c r="B75" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C75" t="s">
         <v>238</v>
@@ -4111,7 +4111,7 @@
         <v>247</v>
       </c>
       <c r="B76" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C76" t="s">
         <v>243</v>
@@ -4122,7 +4122,7 @@
         <v>247</v>
       </c>
       <c r="B77" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C77" t="s">
         <v>252</v>
@@ -4133,7 +4133,7 @@
         <v>247</v>
       </c>
       <c r="B78" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C78" t="s">
         <v>253</v>
@@ -4144,7 +4144,7 @@
         <v>247</v>
       </c>
       <c r="B79" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C79" t="s">
         <v>260</v>
@@ -4166,7 +4166,7 @@
         <v>252</v>
       </c>
       <c r="B81" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C81" t="s">
         <v>264</v>
@@ -4177,7 +4177,7 @@
         <v>252</v>
       </c>
       <c r="B82" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C82" t="s">
         <v>238</v>
@@ -4188,7 +4188,7 @@
         <v>252</v>
       </c>
       <c r="B83" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C83" t="s">
         <v>243</v>
@@ -4199,7 +4199,7 @@
         <v>252</v>
       </c>
       <c r="B84" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C84" t="s">
         <v>247</v>
@@ -4210,7 +4210,7 @@
         <v>252</v>
       </c>
       <c r="B85" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C85" t="s">
         <v>253</v>
@@ -4221,7 +4221,7 @@
         <v>252</v>
       </c>
       <c r="B86" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C86" t="s">
         <v>260</v>
@@ -4243,7 +4243,7 @@
         <v>253</v>
       </c>
       <c r="B88" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C88" t="s">
         <v>264</v>
@@ -4254,7 +4254,7 @@
         <v>253</v>
       </c>
       <c r="B89" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C89" t="s">
         <v>238</v>
@@ -4265,7 +4265,7 @@
         <v>253</v>
       </c>
       <c r="B90" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C90" t="s">
         <v>243</v>
@@ -4276,7 +4276,7 @@
         <v>253</v>
       </c>
       <c r="B91" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C91" t="s">
         <v>247</v>
@@ -4287,7 +4287,7 @@
         <v>253</v>
       </c>
       <c r="B92" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C92" t="s">
         <v>252</v>
@@ -4298,7 +4298,7 @@
         <v>253</v>
       </c>
       <c r="B93" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C93" t="s">
         <v>260</v>
@@ -4320,7 +4320,7 @@
         <v>260</v>
       </c>
       <c r="B95" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C95" t="s">
         <v>264</v>
@@ -4331,7 +4331,7 @@
         <v>260</v>
       </c>
       <c r="B96" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C96" t="s">
         <v>238</v>
@@ -4342,7 +4342,7 @@
         <v>260</v>
       </c>
       <c r="B97" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C97" t="s">
         <v>243</v>
@@ -4353,7 +4353,7 @@
         <v>260</v>
       </c>
       <c r="B98" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C98" t="s">
         <v>247</v>
@@ -4364,7 +4364,7 @@
         <v>260</v>
       </c>
       <c r="B99" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C99" t="s">
         <v>252</v>
@@ -4375,7 +4375,7 @@
         <v>260</v>
       </c>
       <c r="B100" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C100" t="s">
         <v>253</v>
@@ -4383,7 +4383,7 @@
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B101" t="s">
         <v>146</v>
@@ -4394,10 +4394,10 @@
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B102" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C102" t="s">
         <v>173</v>
@@ -4405,10 +4405,10 @@
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B103" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C103" t="s">
         <v>169</v>
@@ -4416,24 +4416,24 @@
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B104" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C104" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B105" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C105" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.2">
@@ -4452,10 +4452,10 @@
         <v>173</v>
       </c>
       <c r="B107" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C107" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.2">
@@ -4463,7 +4463,7 @@
         <v>173</v>
       </c>
       <c r="B108" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C108" t="s">
         <v>169</v>
@@ -4474,10 +4474,10 @@
         <v>173</v>
       </c>
       <c r="B109" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C109" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.2">
@@ -4485,10 +4485,10 @@
         <v>173</v>
       </c>
       <c r="B110" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C110" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.2">
@@ -4507,10 +4507,10 @@
         <v>169</v>
       </c>
       <c r="B112" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C112" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.2">
@@ -4518,7 +4518,7 @@
         <v>169</v>
       </c>
       <c r="B113" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C113" t="s">
         <v>173</v>
@@ -4529,10 +4529,10 @@
         <v>169</v>
       </c>
       <c r="B114" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C114" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.2">
@@ -4540,15 +4540,15 @@
         <v>169</v>
       </c>
       <c r="B115" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C115" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B116" t="s">
         <v>146</v>
@@ -4559,21 +4559,21 @@
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B117" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C117" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B118" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C118" t="s">
         <v>173</v>
@@ -4581,10 +4581,10 @@
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B119" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C119" t="s">
         <v>169</v>
@@ -4592,18 +4592,18 @@
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B120" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C120" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B121" t="s">
         <v>146</v>
@@ -4614,21 +4614,21 @@
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B122" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C122" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B123" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C123" t="s">
         <v>173</v>
@@ -4636,10 +4636,10 @@
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B124" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C124" t="s">
         <v>169</v>
@@ -4647,13 +4647,13 @@
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
+        <v>276</v>
+      </c>
+      <c r="B125" t="s">
+        <v>296</v>
+      </c>
+      <c r="C125" t="s">
         <v>277</v>
-      </c>
-      <c r="B125" t="s">
-        <v>297</v>
-      </c>
-      <c r="C125" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.2">
@@ -4672,7 +4672,7 @@
         <v>178</v>
       </c>
       <c r="B127" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C127" t="s">
         <v>135</v>
@@ -4683,7 +4683,7 @@
         <v>178</v>
       </c>
       <c r="B128" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C128" t="s">
         <v>183</v>
@@ -4694,7 +4694,7 @@
         <v>178</v>
       </c>
       <c r="B129" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C129" t="s">
         <v>187</v>
@@ -4716,7 +4716,7 @@
         <v>135</v>
       </c>
       <c r="B131" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C131" t="s">
         <v>178</v>
@@ -4727,7 +4727,7 @@
         <v>135</v>
       </c>
       <c r="B132" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C132" t="s">
         <v>183</v>
@@ -4738,7 +4738,7 @@
         <v>135</v>
       </c>
       <c r="B133" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C133" t="s">
         <v>187</v>
@@ -4760,7 +4760,7 @@
         <v>183</v>
       </c>
       <c r="B135" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C135" t="s">
         <v>187</v>
@@ -4771,7 +4771,7 @@
         <v>183</v>
       </c>
       <c r="B136" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C136" t="s">
         <v>178</v>
@@ -4782,7 +4782,7 @@
         <v>183</v>
       </c>
       <c r="B137" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C137" t="s">
         <v>135</v>
@@ -4804,7 +4804,7 @@
         <v>187</v>
       </c>
       <c r="B139" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C139" t="s">
         <v>183</v>
@@ -4815,7 +4815,7 @@
         <v>187</v>
       </c>
       <c r="B140" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C140" t="s">
         <v>178</v>
@@ -4826,7 +4826,7 @@
         <v>187</v>
       </c>
       <c r="B141" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C141" t="s">
         <v>135</v>
@@ -4848,10 +4848,10 @@
         <v>191</v>
       </c>
       <c r="B143" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C143" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.2">
@@ -4859,10 +4859,10 @@
         <v>191</v>
       </c>
       <c r="B144" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C144" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.2">
@@ -4870,10 +4870,10 @@
         <v>191</v>
       </c>
       <c r="B145" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C145" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.2">
@@ -4892,10 +4892,10 @@
         <v>196</v>
       </c>
       <c r="B147" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C147" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.2">
@@ -4903,10 +4903,10 @@
         <v>196</v>
       </c>
       <c r="B148" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C148" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.2">
@@ -4914,10 +4914,10 @@
         <v>196</v>
       </c>
       <c r="B149" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C149" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.2">
@@ -4991,7 +4991,7 @@
         <v>201</v>
       </c>
       <c r="B156" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C156" t="s">
         <v>209</v>
@@ -5002,7 +5002,7 @@
         <v>205</v>
       </c>
       <c r="B157" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C157" t="s">
         <v>215</v>
@@ -5010,7 +5010,7 @@
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B158" t="s">
         <v>146</v>
@@ -5021,10 +5021,10 @@
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B159" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C159" t="s">
         <v>191</v>
@@ -5032,10 +5032,10 @@
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B160" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C160" t="s">
         <v>196</v>
@@ -5043,7 +5043,7 @@
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B161" t="s">
         <v>146</v>
@@ -5054,10 +5054,10 @@
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B162" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C162" t="s">
         <v>191</v>
@@ -5065,10 +5065,10 @@
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B163" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C163" t="s">
         <v>196</v>
@@ -5076,7 +5076,7 @@
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B164" t="s">
         <v>146</v>
@@ -5087,10 +5087,10 @@
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B165" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C165" t="s">
         <v>191</v>
@@ -5098,10 +5098,10 @@
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B166" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C166" t="s">
         <v>196</v>
@@ -5134,7 +5134,7 @@
         <v>209</v>
       </c>
       <c r="B169" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C169" t="s">
         <v>201</v>
@@ -5145,7 +5145,7 @@
         <v>215</v>
       </c>
       <c r="B170" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C170" t="s">
         <v>205</v>
@@ -5251,10 +5251,10 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C3" s="9" t="s">
         <v>110</v>
@@ -5278,10 +5278,10 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="9" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>110</v>
@@ -5313,10 +5313,10 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>110</v>
@@ -5348,10 +5348,10 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>110</v>
@@ -5373,7 +5373,7 @@
       </c>
       <c r="I6" s="9"/>
       <c r="J6" s="9" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="K6" s="9"/>
       <c r="L6" s="9"/>
@@ -5381,10 +5381,10 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>110</v>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="I7" s="9"/>
       <c r="J7" s="9" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="K7" s="9"/>
       <c r="L7" s="9"/>
@@ -5449,10 +5449,10 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>110</v>
@@ -5473,23 +5473,23 @@
         <v>243</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="J9" s="9" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="K9" s="9"/>
       <c r="L9" s="9" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="M9" s="9"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>110</v>
@@ -5510,23 +5510,23 @@
         <v>260</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="K10" s="9" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="L10" s="9"/>
       <c r="M10" s="9"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="9" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>110</v>
@@ -5553,17 +5553,17 @@
         <v>144</v>
       </c>
       <c r="K11" s="9" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="L11" s="9"/>
       <c r="M11" s="9"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>110</v>
@@ -5581,16 +5581,16 @@
         <v>224</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="J12" s="9" t="s">
         <v>144</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="L12" s="9"/>
       <c r="M12" s="9"/>

</xml_diff>

<commit_message>
Bumper vs bumper OP exclusivity from spreadsheet; show same-category EXCLUDES in UI
- Regenerate configMatrix from updated Excel (bidirectional EXCLUDES for bumpers)
- canSelectPart: treat EXCLUDES within any shared category like wheelbase (visible to switch)
- enforceRules still removes conflicting body parts when both would apply

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Configurator_Data.xlsx
+++ b/Configurator_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samrosati/Documents/upt-configurator-test-repo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{634E7B65-7A0D-C243-8B75-21442EBD5191}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{275E79D3-78CB-5440-B4C8-C7D5DDA6D9CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1130" uniqueCount="371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1142" uniqueCount="371">
   <si>
     <t>3D CONFIGURATOR - Customer Data Template</t>
   </si>
@@ -3266,7 +3266,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D170"/>
+  <dimension ref="A1:D174"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -4955,18 +4955,18 @@
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
-        <v>141</v>
+        <v>53</v>
       </c>
       <c r="B153" t="s">
-        <v>146</v>
+        <v>296</v>
       </c>
       <c r="C153" t="s">
-        <v>110</v>
+        <v>201</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
-        <v>201</v>
+        <v>141</v>
       </c>
       <c r="B154" t="s">
         <v>146</v>
@@ -4977,13 +4977,13 @@
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
+        <v>141</v>
+      </c>
+      <c r="B155" t="s">
+        <v>296</v>
+      </c>
+      <c r="C155" t="s">
         <v>205</v>
-      </c>
-      <c r="B155" t="s">
-        <v>146</v>
-      </c>
-      <c r="C155" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.2">
@@ -4991,163 +4991,207 @@
         <v>201</v>
       </c>
       <c r="B156" t="s">
-        <v>296</v>
+        <v>146</v>
       </c>
       <c r="C156" t="s">
-        <v>209</v>
+        <v>110</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B157" t="s">
         <v>296</v>
       </c>
       <c r="C157" t="s">
-        <v>215</v>
+        <v>53</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
-        <v>282</v>
+        <v>205</v>
       </c>
       <c r="B158" t="s">
         <v>146</v>
       </c>
       <c r="C158" t="s">
-        <v>48</v>
+        <v>110</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
-        <v>282</v>
+        <v>205</v>
       </c>
       <c r="B159" t="s">
         <v>296</v>
       </c>
       <c r="C159" t="s">
-        <v>191</v>
+        <v>141</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
-        <v>282</v>
+        <v>201</v>
       </c>
       <c r="B160" t="s">
         <v>296</v>
       </c>
       <c r="C160" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
-        <v>287</v>
+        <v>205</v>
       </c>
       <c r="B161" t="s">
-        <v>146</v>
+        <v>296</v>
       </c>
       <c r="C161" t="s">
-        <v>48</v>
+        <v>215</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="B162" t="s">
-        <v>296</v>
+        <v>146</v>
       </c>
       <c r="C162" t="s">
-        <v>191</v>
+        <v>48</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="B163" t="s">
         <v>296</v>
       </c>
       <c r="C163" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="B164" t="s">
-        <v>146</v>
+        <v>296</v>
       </c>
       <c r="C164" t="s">
-        <v>48</v>
+        <v>196</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B165" t="s">
-        <v>296</v>
+        <v>146</v>
       </c>
       <c r="C165" t="s">
-        <v>191</v>
+        <v>48</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B166" t="s">
         <v>296</v>
       </c>
       <c r="C166" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
-        <v>209</v>
+        <v>287</v>
       </c>
       <c r="B167" t="s">
-        <v>146</v>
+        <v>296</v>
       </c>
       <c r="C167" t="s">
-        <v>110</v>
+        <v>196</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
-        <v>215</v>
+        <v>288</v>
       </c>
       <c r="B168" t="s">
         <v>146</v>
       </c>
       <c r="C168" t="s">
-        <v>110</v>
+        <v>48</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
-        <v>209</v>
+        <v>288</v>
       </c>
       <c r="B169" t="s">
         <v>296</v>
       </c>
       <c r="C169" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
+        <v>288</v>
+      </c>
+      <c r="B170" t="s">
+        <v>296</v>
+      </c>
+      <c r="C170" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="171" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A171" t="s">
+        <v>209</v>
+      </c>
+      <c r="B171" t="s">
+        <v>146</v>
+      </c>
+      <c r="C171" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="172" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A172" t="s">
         <v>215</v>
       </c>
-      <c r="B170" t="s">
-        <v>296</v>
-      </c>
-      <c r="C170" t="s">
+      <c r="B172" t="s">
+        <v>146</v>
+      </c>
+      <c r="C172" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="173" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A173" t="s">
+        <v>209</v>
+      </c>
+      <c r="B173" t="s">
+        <v>296</v>
+      </c>
+      <c r="C173" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="174" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A174" t="s">
+        <v>215</v>
+      </c>
+      <c r="B174" t="s">
+        <v>296</v>
+      </c>
+      <c r="C174" t="s">
         <v>205</v>
       </c>
     </row>

</xml_diff>

<commit_message>
SXS preset with fenders; split Cargo Bike and Cargo Bike Long presets; rules for long topbody
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Configurator_Data.xlsx
+++ b/Configurator_Data.xlsx
@@ -2026,7 +2026,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D174"/>
+  <dimension ref="A1:D179"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2066,6 +2066,9 @@
       <c r="C3" t="str">
         <v>block-single</v>
       </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -2077,6 +2080,9 @@
       <c r="C4" t="str">
         <v>wb-1330</v>
       </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -2088,6 +2094,9 @@
       <c r="C5" t="str">
         <v>block-single</v>
       </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -2099,6 +2108,9 @@
       <c r="C6" t="str">
         <v>wb-1130</v>
       </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -2110,6 +2122,9 @@
       <c r="C7" t="str">
         <v>wb-1130</v>
       </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -2121,6 +2136,9 @@
       <c r="C8" t="str">
         <v>motor-a-1330</v>
       </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -2132,6 +2150,9 @@
       <c r="C9" t="str">
         <v>wb-1330</v>
       </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -2143,6 +2164,9 @@
       <c r="C10" t="str">
         <v>motor-a-1130</v>
       </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -2154,6 +2178,9 @@
       <c r="C11" t="str">
         <v>motor-a-1130</v>
       </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -2165,6 +2192,9 @@
       <c r="C12" t="str">
         <v>tire-offroad-1130</v>
       </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -2176,6 +2206,9 @@
       <c r="C13" t="str">
         <v>tire-urban-1330</v>
       </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -2187,6 +2220,9 @@
       <c r="C14" t="str">
         <v>tire-offroad-1330</v>
       </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -2198,6 +2234,9 @@
       <c r="C15" t="str">
         <v>motor-a-1130</v>
       </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -2209,6 +2248,9 @@
       <c r="C16" t="str">
         <v>tire-urban-1130</v>
       </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -2220,6 +2262,9 @@
       <c r="C17" t="str">
         <v>tire-urban-1330</v>
       </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -2231,6 +2276,9 @@
       <c r="C18" t="str">
         <v>tire-offroad-1330</v>
       </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -2242,6 +2290,9 @@
       <c r="C19" t="str">
         <v>motor-a-1330</v>
       </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -2253,6 +2304,9 @@
       <c r="C20" t="str">
         <v>tire-urban-1130</v>
       </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -2264,6 +2318,9 @@
       <c r="C21" t="str">
         <v>tire-offroad-1130</v>
       </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -2275,6 +2332,9 @@
       <c r="C22" t="str">
         <v>tire-offroad-1330</v>
       </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -2286,6 +2346,9 @@
       <c r="C23" t="str">
         <v>motor-a-1330</v>
       </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -2297,6 +2360,9 @@
       <c r="C24" t="str">
         <v>tire-urban-1130</v>
       </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -2308,6 +2374,9 @@
       <c r="C25" t="str">
         <v>tire-offroad-1130</v>
       </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -2319,6 +2388,9 @@
       <c r="C26" t="str">
         <v>tire-urban-1330</v>
       </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -2330,6 +2402,9 @@
       <c r="C27" t="str">
         <v>block-single</v>
       </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -2341,6 +2416,9 @@
       <c r="C28" t="str">
         <v>column-65</v>
       </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -2352,6 +2430,9 @@
       <c r="C29" t="str">
         <v>column-65-L</v>
       </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -2363,6 +2444,9 @@
       <c r="C30" t="str">
         <v>column-45</v>
       </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -2374,6 +2458,9 @@
       <c r="C31" t="str">
         <v>column-cycling</v>
       </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -2385,6 +2472,9 @@
       <c r="C32" t="str">
         <v>block-single</v>
       </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -2396,6 +2486,9 @@
       <c r="C33" t="str">
         <v>column-90</v>
       </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -2407,6 +2500,9 @@
       <c r="C34" t="str">
         <v>column-65-L</v>
       </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -2418,6 +2514,9 @@
       <c r="C35" t="str">
         <v>column-45</v>
       </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -2429,6 +2528,9 @@
       <c r="C36" t="str">
         <v>column-cycling</v>
       </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -2440,6 +2542,9 @@
       <c r="C37" t="str">
         <v>block-single</v>
       </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -2451,6 +2556,9 @@
       <c r="C38" t="str">
         <v>column-90</v>
       </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -2462,6 +2570,9 @@
       <c r="C39" t="str">
         <v>column-65</v>
       </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -2473,6 +2584,9 @@
       <c r="C40" t="str">
         <v>column-45</v>
       </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -2484,6 +2598,9 @@
       <c r="C41" t="str">
         <v>column-cycling</v>
       </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -2495,6 +2612,9 @@
       <c r="C42" t="str">
         <v>block-single</v>
       </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -2506,6 +2626,9 @@
       <c r="C43" t="str">
         <v>column-90</v>
       </c>
+      <c r="D43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -2517,6 +2640,9 @@
       <c r="C44" t="str">
         <v>column-65</v>
       </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -2528,6 +2654,9 @@
       <c r="C45" t="str">
         <v>column-65-L</v>
       </c>
+      <c r="D45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -2539,6 +2668,9 @@
       <c r="C46" t="str">
         <v>column-cycling</v>
       </c>
+      <c r="D46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -2550,6 +2682,9 @@
       <c r="C47" t="str">
         <v>block-single</v>
       </c>
+      <c r="D47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -2561,6 +2696,9 @@
       <c r="C48" t="str">
         <v>column-90</v>
       </c>
+      <c r="D48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -2572,6 +2710,9 @@
       <c r="C49" t="str">
         <v>column-65</v>
       </c>
+      <c r="D49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -2583,6 +2724,9 @@
       <c r="C50" t="str">
         <v>column-65-L</v>
       </c>
+      <c r="D50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -2594,6 +2738,9 @@
       <c r="C51" t="str">
         <v>column-45</v>
       </c>
+      <c r="D51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -2605,6 +2752,9 @@
       <c r="C52" t="str">
         <v>control-handlebarrev</v>
       </c>
+      <c r="D52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -2616,6 +2766,9 @@
       <c r="C53" t="str">
         <v>handle-bar-65</v>
       </c>
+      <c r="D53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -2627,6 +2780,9 @@
       <c r="C54" t="str">
         <v>handle-bar-65-sxs</v>
       </c>
+      <c r="D54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -2638,6 +2794,9 @@
       <c r="C55" t="str">
         <v>handle-bar-65-L</v>
       </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -2649,6 +2808,9 @@
       <c r="C56" t="str">
         <v>handle-sw-45</v>
       </c>
+      <c r="D56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -2660,6 +2822,9 @@
       <c r="C57" t="str">
         <v>handle-sw-65</v>
       </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -2671,6 +2836,9 @@
       <c r="C58" t="str">
         <v>handle-sw-65-sxs</v>
       </c>
+      <c r="D58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -2682,6 +2850,9 @@
       <c r="C59" t="str">
         <v>column-65</v>
       </c>
+      <c r="D59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -2693,6 +2864,9 @@
       <c r="C60" t="str">
         <v>handle-bar-90-rev</v>
       </c>
+      <c r="D60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -2704,6 +2878,9 @@
       <c r="C61" t="str">
         <v>handle-bar-65-sxs</v>
       </c>
+      <c r="D61" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -2715,6 +2892,9 @@
       <c r="C62" t="str">
         <v>handle-bar-65-L</v>
       </c>
+      <c r="D62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -2726,6 +2906,9 @@
       <c r="C63" t="str">
         <v>handle-sw-45</v>
       </c>
+      <c r="D63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -2737,6 +2920,9 @@
       <c r="C64" t="str">
         <v>handle-sw-65</v>
       </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -2748,6 +2934,9 @@
       <c r="C65" t="str">
         <v>handle-sw-65-sxs</v>
       </c>
+      <c r="D65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -2759,6 +2948,9 @@
       <c r="C66" t="str">
         <v>column-65</v>
       </c>
+      <c r="D66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -2770,6 +2962,9 @@
       <c r="C67" t="str">
         <v>handle-bar-90-rev</v>
       </c>
+      <c r="D67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -2781,6 +2976,9 @@
       <c r="C68" t="str">
         <v>handle-bar-65</v>
       </c>
+      <c r="D68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -2792,6 +2990,9 @@
       <c r="C69" t="str">
         <v>handle-bar-65-L</v>
       </c>
+      <c r="D69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -2803,6 +3004,9 @@
       <c r="C70" t="str">
         <v>handle-sw-45</v>
       </c>
+      <c r="D70" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -2814,6 +3018,9 @@
       <c r="C71" t="str">
         <v>handle-sw-65</v>
       </c>
+      <c r="D71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -2825,6 +3032,9 @@
       <c r="C72" t="str">
         <v>handle-sw-65-sxs</v>
       </c>
+      <c r="D72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -2836,6 +3046,9 @@
       <c r="C73" t="str">
         <v>column-65-L</v>
       </c>
+      <c r="D73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -2847,6 +3060,9 @@
       <c r="C74" t="str">
         <v>handle-bar-90-rev</v>
       </c>
+      <c r="D74" t="str">
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -2858,6 +3074,9 @@
       <c r="C75" t="str">
         <v>handle-bar-65</v>
       </c>
+      <c r="D75" t="str">
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -2869,6 +3088,9 @@
       <c r="C76" t="str">
         <v>handle-bar-65-sxs</v>
       </c>
+      <c r="D76" t="str">
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -2880,6 +3102,9 @@
       <c r="C77" t="str">
         <v>handle-sw-45</v>
       </c>
+      <c r="D77" t="str">
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -2891,6 +3116,9 @@
       <c r="C78" t="str">
         <v>handle-sw-65</v>
       </c>
+      <c r="D78" t="str">
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -2902,6 +3130,9 @@
       <c r="C79" t="str">
         <v>handle-sw-65-sxs</v>
       </c>
+      <c r="D79" t="str">
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -2913,6 +3144,9 @@
       <c r="C80" t="str">
         <v>column-45</v>
       </c>
+      <c r="D80" t="str">
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -2924,6 +3158,9 @@
       <c r="C81" t="str">
         <v>handle-bar-90-rev</v>
       </c>
+      <c r="D81" t="str">
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -2935,6 +3172,9 @@
       <c r="C82" t="str">
         <v>handle-bar-65</v>
       </c>
+      <c r="D82" t="str">
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -2946,6 +3186,9 @@
       <c r="C83" t="str">
         <v>handle-bar-65-sxs</v>
       </c>
+      <c r="D83" t="str">
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -2957,6 +3200,9 @@
       <c r="C84" t="str">
         <v>handle-bar-65-L</v>
       </c>
+      <c r="D84" t="str">
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -2968,6 +3214,9 @@
       <c r="C85" t="str">
         <v>handle-sw-65</v>
       </c>
+      <c r="D85" t="str">
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -2979,6 +3228,9 @@
       <c r="C86" t="str">
         <v>handle-sw-65-sxs</v>
       </c>
+      <c r="D86" t="str">
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -2990,6 +3242,9 @@
       <c r="C87" t="str">
         <v>column-65</v>
       </c>
+      <c r="D87" t="str">
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -3001,6 +3256,9 @@
       <c r="C88" t="str">
         <v>handle-bar-90-rev</v>
       </c>
+      <c r="D88" t="str">
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -3012,6 +3270,9 @@
       <c r="C89" t="str">
         <v>handle-bar-65</v>
       </c>
+      <c r="D89" t="str">
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -3023,6 +3284,9 @@
       <c r="C90" t="str">
         <v>handle-bar-65-sxs</v>
       </c>
+      <c r="D90" t="str">
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -3034,6 +3298,9 @@
       <c r="C91" t="str">
         <v>handle-bar-65-L</v>
       </c>
+      <c r="D91" t="str">
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -3045,6 +3312,9 @@
       <c r="C92" t="str">
         <v>handle-sw-45</v>
       </c>
+      <c r="D92" t="str">
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -3056,6 +3326,9 @@
       <c r="C93" t="str">
         <v>handle-sw-65-sxs</v>
       </c>
+      <c r="D93" t="str">
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -3067,6 +3340,9 @@
       <c r="C94" t="str">
         <v>column-65</v>
       </c>
+      <c r="D94" t="str">
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
@@ -3078,6 +3354,9 @@
       <c r="C95" t="str">
         <v>handle-bar-90-rev</v>
       </c>
+      <c r="D95" t="str">
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
@@ -3089,6 +3368,9 @@
       <c r="C96" t="str">
         <v>handle-bar-65</v>
       </c>
+      <c r="D96" t="str">
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
@@ -3100,6 +3382,9 @@
       <c r="C97" t="str">
         <v>handle-bar-65-sxs</v>
       </c>
+      <c r="D97" t="str">
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
@@ -3111,6 +3396,9 @@
       <c r="C98" t="str">
         <v>handle-bar-65-L</v>
       </c>
+      <c r="D98" t="str">
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
@@ -3122,6 +3410,9 @@
       <c r="C99" t="str">
         <v>handle-sw-45</v>
       </c>
+      <c r="D99" t="str">
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
@@ -3133,6 +3424,9 @@
       <c r="C100" t="str">
         <v>handle-sw-65</v>
       </c>
+      <c r="D100" t="str">
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
@@ -3144,6 +3438,9 @@
       <c r="C101" t="str">
         <v>block-single</v>
       </c>
+      <c r="D101" t="str">
+        <v/>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
@@ -3155,6 +3452,9 @@
       <c r="C102" t="str">
         <v>seat-bucket</v>
       </c>
+      <c r="D102" t="str">
+        <v/>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
@@ -3166,6 +3466,9 @@
       <c r="C103" t="str">
         <v>seat-full</v>
       </c>
+      <c r="D103" t="str">
+        <v/>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
@@ -3177,6 +3480,9 @@
       <c r="C104" t="str">
         <v>seat-sxs</v>
       </c>
+      <c r="D104" t="str">
+        <v/>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
@@ -3188,6 +3494,9 @@
       <c r="C105" t="str">
         <v>seat-bike</v>
       </c>
+      <c r="D105" t="str">
+        <v/>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
@@ -3199,6 +3508,9 @@
       <c r="C106" t="str">
         <v>block-single</v>
       </c>
+      <c r="D106" t="str">
+        <v/>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
@@ -3210,6 +3522,9 @@
       <c r="C107" t="str">
         <v>seat-lean</v>
       </c>
+      <c r="D107" t="str">
+        <v/>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
@@ -3221,6 +3536,9 @@
       <c r="C108" t="str">
         <v>seat-full</v>
       </c>
+      <c r="D108" t="str">
+        <v/>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
@@ -3232,6 +3550,9 @@
       <c r="C109" t="str">
         <v>seat-sxs</v>
       </c>
+      <c r="D109" t="str">
+        <v/>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
@@ -3243,6 +3564,9 @@
       <c r="C110" t="str">
         <v>seat-bike</v>
       </c>
+      <c r="D110" t="str">
+        <v/>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
@@ -3254,6 +3578,9 @@
       <c r="C111" t="str">
         <v>block-single</v>
       </c>
+      <c r="D111" t="str">
+        <v/>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
@@ -3265,6 +3592,9 @@
       <c r="C112" t="str">
         <v>seat-lean</v>
       </c>
+      <c r="D112" t="str">
+        <v/>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
@@ -3276,6 +3606,9 @@
       <c r="C113" t="str">
         <v>seat-bucket</v>
       </c>
+      <c r="D113" t="str">
+        <v/>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
@@ -3287,6 +3620,9 @@
       <c r="C114" t="str">
         <v>seat-sxs</v>
       </c>
+      <c r="D114" t="str">
+        <v/>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
@@ -3298,6 +3634,9 @@
       <c r="C115" t="str">
         <v>seat-bike</v>
       </c>
+      <c r="D115" t="str">
+        <v/>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
@@ -3309,6 +3648,9 @@
       <c r="C116" t="str">
         <v>block-single</v>
       </c>
+      <c r="D116" t="str">
+        <v/>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
@@ -3320,6 +3662,9 @@
       <c r="C117" t="str">
         <v>seat-lean</v>
       </c>
+      <c r="D117" t="str">
+        <v/>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
@@ -3331,6 +3676,9 @@
       <c r="C118" t="str">
         <v>seat-bucket</v>
       </c>
+      <c r="D118" t="str">
+        <v/>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
@@ -3342,6 +3690,9 @@
       <c r="C119" t="str">
         <v>seat-full</v>
       </c>
+      <c r="D119" t="str">
+        <v/>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
@@ -3353,6 +3704,9 @@
       <c r="C120" t="str">
         <v>seat-bike</v>
       </c>
+      <c r="D120" t="str">
+        <v/>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
@@ -3364,6 +3718,9 @@
       <c r="C121" t="str">
         <v>block-single</v>
       </c>
+      <c r="D121" t="str">
+        <v/>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
@@ -3375,6 +3732,9 @@
       <c r="C122" t="str">
         <v>seat-lean</v>
       </c>
+      <c r="D122" t="str">
+        <v/>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
@@ -3386,6 +3746,9 @@
       <c r="C123" t="str">
         <v>seat-bucket</v>
       </c>
+      <c r="D123" t="str">
+        <v/>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
@@ -3397,6 +3760,9 @@
       <c r="C124" t="str">
         <v>seat-full</v>
       </c>
+      <c r="D124" t="str">
+        <v/>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
@@ -3408,6 +3774,9 @@
       <c r="C125" t="str">
         <v>seat-sxs</v>
       </c>
+      <c r="D125" t="str">
+        <v/>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
@@ -3419,6 +3788,9 @@
       <c r="C126" t="str">
         <v>block-single</v>
       </c>
+      <c r="D126" t="str">
+        <v/>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
@@ -3430,6 +3802,9 @@
       <c r="C127" t="str">
         <v>body-sidesteplg</v>
       </c>
+      <c r="D127" t="str">
+        <v/>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
@@ -3441,6 +3816,9 @@
       <c r="C128" t="str">
         <v>body-flatbedsm</v>
       </c>
+      <c r="D128" t="str">
+        <v/>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
@@ -3452,6 +3830,9 @@
       <c r="C129" t="str">
         <v>body-flatbedlg</v>
       </c>
+      <c r="D129" t="str">
+        <v/>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
@@ -3463,6 +3844,9 @@
       <c r="C130" t="str">
         <v>block-single</v>
       </c>
+      <c r="D130" t="str">
+        <v/>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
@@ -3474,6 +3858,9 @@
       <c r="C131" t="str">
         <v>body-sidestepsm</v>
       </c>
+      <c r="D131" t="str">
+        <v/>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
@@ -3485,6 +3872,9 @@
       <c r="C132" t="str">
         <v>body-flatbedsm</v>
       </c>
+      <c r="D132" t="str">
+        <v/>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
@@ -3496,6 +3886,9 @@
       <c r="C133" t="str">
         <v>body-flatbedlg</v>
       </c>
+      <c r="D133" t="str">
+        <v/>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
@@ -3507,6 +3900,9 @@
       <c r="C134" t="str">
         <v>block-single</v>
       </c>
+      <c r="D134" t="str">
+        <v/>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
@@ -3518,6 +3914,9 @@
       <c r="C135" t="str">
         <v>body-flatbedlg</v>
       </c>
+      <c r="D135" t="str">
+        <v/>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
@@ -3529,6 +3928,9 @@
       <c r="C136" t="str">
         <v>body-sidestepsm</v>
       </c>
+      <c r="D136" t="str">
+        <v/>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
@@ -3540,6 +3942,9 @@
       <c r="C137" t="str">
         <v>body-sidesteplg</v>
       </c>
+      <c r="D137" t="str">
+        <v/>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
@@ -3551,6 +3956,9 @@
       <c r="C138" t="str">
         <v>block-single</v>
       </c>
+      <c r="D138" t="str">
+        <v/>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
@@ -3562,6 +3970,9 @@
       <c r="C139" t="str">
         <v>body-flatbedsm</v>
       </c>
+      <c r="D139" t="str">
+        <v/>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
@@ -3573,6 +3984,9 @@
       <c r="C140" t="str">
         <v>body-sidestepsm</v>
       </c>
+      <c r="D140" t="str">
+        <v/>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
@@ -3584,6 +3998,9 @@
       <c r="C141" t="str">
         <v>body-sidesteplg</v>
       </c>
+      <c r="D141" t="str">
+        <v/>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
@@ -3595,6 +4012,9 @@
       <c r="C142" t="str">
         <v>body-fenders</v>
       </c>
+      <c r="D142" t="str">
+        <v/>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
@@ -3606,6 +4026,9 @@
       <c r="C143" t="str">
         <v>topbody-lsv</v>
       </c>
+      <c r="D143" t="str">
+        <v/>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
@@ -3617,6 +4040,9 @@
       <c r="C144" t="str">
         <v>topbody-golf</v>
       </c>
+      <c r="D144" t="str">
+        <v/>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
@@ -3628,6 +4054,9 @@
       <c r="C145" t="str">
         <v>topbody-cargobike</v>
       </c>
+      <c r="D145" t="str">
+        <v/>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
@@ -3639,6 +4068,9 @@
       <c r="C146" t="str">
         <v>body-fenders</v>
       </c>
+      <c r="D146" t="str">
+        <v/>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
@@ -3650,6 +4082,9 @@
       <c r="C147" t="str">
         <v>topbody-lsv</v>
       </c>
+      <c r="D147" t="str">
+        <v/>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
@@ -3661,6 +4096,9 @@
       <c r="C148" t="str">
         <v>topbody-golf</v>
       </c>
+      <c r="D148" t="str">
+        <v/>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
@@ -3672,6 +4110,9 @@
       <c r="C149" t="str">
         <v>topbody-cargobike</v>
       </c>
+      <c r="D149" t="str">
+        <v/>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
@@ -3683,6 +4124,9 @@
       <c r="C150" t="str">
         <v>block-single</v>
       </c>
+      <c r="D150" t="str">
+        <v/>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
@@ -3694,6 +4138,9 @@
       <c r="C151" t="str">
         <v>body-sidesteplg</v>
       </c>
+      <c r="D151" t="str">
+        <v/>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="str">
@@ -3705,6 +4152,9 @@
       <c r="C152" t="str">
         <v>block-single</v>
       </c>
+      <c r="D152" t="str">
+        <v/>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="str">
@@ -3716,6 +4166,9 @@
       <c r="C153" t="str">
         <v>body-frontbumperop</v>
       </c>
+      <c r="D153" t="str">
+        <v/>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="str">
@@ -3727,6 +4180,9 @@
       <c r="C154" t="str">
         <v>block-single</v>
       </c>
+      <c r="D154" t="str">
+        <v/>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="str">
@@ -3738,6 +4194,9 @@
       <c r="C155" t="str">
         <v>body-rearbumperop</v>
       </c>
+      <c r="D155" t="str">
+        <v/>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="str">
@@ -3749,6 +4208,9 @@
       <c r="C156" t="str">
         <v>block-single</v>
       </c>
+      <c r="D156" t="str">
+        <v/>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="str">
@@ -3760,6 +4222,9 @@
       <c r="C157" t="str">
         <v>body-frontbumper</v>
       </c>
+      <c r="D157" t="str">
+        <v/>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="str">
@@ -3771,6 +4236,9 @@
       <c r="C158" t="str">
         <v>block-single</v>
       </c>
+      <c r="D158" t="str">
+        <v/>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
@@ -3782,6 +4250,9 @@
       <c r="C159" t="str">
         <v>body-rearbumper</v>
       </c>
+      <c r="D159" t="str">
+        <v/>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
@@ -3793,6 +4264,9 @@
       <c r="C160" t="str">
         <v>acc-winch</v>
       </c>
+      <c r="D160" t="str">
+        <v/>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
@@ -3804,6 +4278,9 @@
       <c r="C161" t="str">
         <v>acc-hitch</v>
       </c>
+      <c r="D161" t="str">
+        <v/>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
@@ -3815,6 +4292,9 @@
       <c r="C162" t="str">
         <v>body-fenders</v>
       </c>
+      <c r="D162" t="str">
+        <v/>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
@@ -3826,6 +4306,9 @@
       <c r="C163" t="str">
         <v>body-frontrack</v>
       </c>
+      <c r="D163" t="str">
+        <v/>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
@@ -3837,6 +4320,9 @@
       <c r="C164" t="str">
         <v>body-rearack</v>
       </c>
+      <c r="D164" t="str">
+        <v/>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
@@ -3848,6 +4334,9 @@
       <c r="C165" t="str">
         <v>body-fenders</v>
       </c>
+      <c r="D165" t="str">
+        <v/>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
@@ -3859,6 +4348,9 @@
       <c r="C166" t="str">
         <v>body-frontrack</v>
       </c>
+      <c r="D166" t="str">
+        <v/>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
@@ -3870,6 +4362,9 @@
       <c r="C167" t="str">
         <v>body-rearack</v>
       </c>
+      <c r="D167" t="str">
+        <v/>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
@@ -3881,6 +4376,9 @@
       <c r="C168" t="str">
         <v>body-fenders</v>
       </c>
+      <c r="D168" t="str">
+        <v/>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
@@ -3892,6 +4390,9 @@
       <c r="C169" t="str">
         <v>body-frontrack</v>
       </c>
+      <c r="D169" t="str">
+        <v/>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
@@ -3903,6 +4404,9 @@
       <c r="C170" t="str">
         <v>body-rearack</v>
       </c>
+      <c r="D170" t="str">
+        <v/>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
@@ -3914,6 +4418,9 @@
       <c r="C171" t="str">
         <v>block-single</v>
       </c>
+      <c r="D171" t="str">
+        <v/>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
@@ -3925,6 +4432,9 @@
       <c r="C172" t="str">
         <v>block-single</v>
       </c>
+      <c r="D172" t="str">
+        <v/>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
@@ -3936,6 +4446,9 @@
       <c r="C173" t="str">
         <v>body-frontbumperop</v>
       </c>
+      <c r="D173" t="str">
+        <v/>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
@@ -3947,18 +4460,90 @@
       <c r="C174" t="str">
         <v>body-rearbumperop</v>
       </c>
+      <c r="D174" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="str">
+        <v>body-frontrack</v>
+      </c>
+      <c r="B175" t="str">
+        <v>EXCLUDES</v>
+      </c>
+      <c r="C175" t="str">
+        <v>topbody-cargobike-l</v>
+      </c>
+      <c r="D175" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="str">
+        <v>body-rearack</v>
+      </c>
+      <c r="B176" t="str">
+        <v>EXCLUDES</v>
+      </c>
+      <c r="C176" t="str">
+        <v>topbody-cargobike-l</v>
+      </c>
+      <c r="D176" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="str">
+        <v>topbody-cargobike-l</v>
+      </c>
+      <c r="B177" t="str">
+        <v>REQUIRES</v>
+      </c>
+      <c r="C177" t="str">
+        <v>body-fenders</v>
+      </c>
+      <c r="D177" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="str">
+        <v>topbody-cargobike-l</v>
+      </c>
+      <c r="B178" t="str">
+        <v>EXCLUDES</v>
+      </c>
+      <c r="C178" t="str">
+        <v>body-frontrack</v>
+      </c>
+      <c r="D178" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>topbody-cargobike-l</v>
+      </c>
+      <c r="B179" t="str">
+        <v>EXCLUDES</v>
+      </c>
+      <c r="C179" t="str">
+        <v>body-rearack</v>
+      </c>
+      <c r="D179" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D174"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D179"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4317,7 +4902,7 @@
         <v>seat-sxs</v>
       </c>
       <c r="J9" t="str">
-        <v>body-flatbedlg, body-frontbumper</v>
+        <v>body-sidesteplg, body-fenders, body-frontbumper</v>
       </c>
       <c r="K9" t="str">
         <v/>
@@ -4452,9 +5037,50 @@
         <v/>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Cargo Bike Long</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Long-wheelbase cargo bike with extended top</v>
+      </c>
+      <c r="C13" t="str">
+        <v>block-single</v>
+      </c>
+      <c r="D13" t="str">
+        <v>wb-1330</v>
+      </c>
+      <c r="E13" t="str">
+        <v>tire-cargobike-1330</v>
+      </c>
+      <c r="F13" t="str">
+        <v>motor-a-1330</v>
+      </c>
+      <c r="G13" t="str">
+        <v>column-cargobike-l</v>
+      </c>
+      <c r="H13" t="str">
+        <v>handle-cargobike-l</v>
+      </c>
+      <c r="I13" t="str">
+        <v>seat-cargo-bike</v>
+      </c>
+      <c r="J13" t="str">
+        <v>body-sidesteplg, body-fenders, body-frontbumper, body-rearbumper</v>
+      </c>
+      <c r="K13" t="str">
+        <v>topbody-cargobike-l</v>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>